<commit_message>
DEV: Misc bug fixes.
</commit_message>
<xml_diff>
--- a/Data/IpAddressConditionalFormattingTemplate.xlsx
+++ b/Data/IpAddressConditionalFormattingTemplate.xlsx
@@ -195,7 +195,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="120">
+  <dxfs count="145">
     <dxf>
       <fill>
         <patternFill>
@@ -262,6 +262,181 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
     <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <fill>
         <patternFill>
@@ -1529,31 +1704,31 @@
     <row r="78" ht="15" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="A:A">
-    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="115">
+    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="140">
       <formula>NOT(ISERROR(SEARCH("microsoft",A1)))</formula>
     </cfRule>
-    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="116">
+    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="141">
       <formula>NOT(ISERROR(SEARCH("proofpoint",A1)))</formula>
     </cfRule>
-    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="117">
+    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="142">
       <formula>NOT(ISERROR(SEARCH(" vpn",A1)))</formula>
     </cfRule>
-    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="117">
+    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="142">
       <formula>NOT(ISERROR(SEARCH(" tor",A1)))</formula>
     </cfRule>
-    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="117">
+    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="142">
       <formula>NOT(ISERROR(SEARCH(" proxy",A1)))</formula>
     </cfRule>
-    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="118">
+    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="143">
       <formula>NOT(ISERROR(SEARCH(" hosting",A1)))</formula>
     </cfRule>
-    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="118">
+    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="143">
       <formula>NOT(ISERROR(SEARCH(" cloud",A1)))</formula>
     </cfRule>
-    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="118">
+    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="143">
       <formula>NOT(ISERROR(SEARCH(" datacenter",A1)))</formula>
     </cfRule>
-    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="119">
+    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="144">
       <formula>NOT(ISERROR(SEARCH("mobile",A1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
DEV: Updated documentation. FEATURE: Made Get-IRTTenantOIDC public. Added ability to search domain, return tenant id.
</commit_message>
<xml_diff>
--- a/Data/IpAddressConditionalFormattingTemplate.xlsx
+++ b/Data/IpAddressConditionalFormattingTemplate.xlsx
@@ -195,7 +195,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="145">
+  <dxfs count="155">
     <dxf>
       <fill>
         <patternFill>
@@ -262,6 +262,76 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
     <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <fill>
         <patternFill>
@@ -1704,31 +1774,31 @@
     <row r="78" ht="15" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="A:A">
-    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="140">
+    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="150">
       <formula>NOT(ISERROR(SEARCH("microsoft",A1)))</formula>
     </cfRule>
-    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="141">
+    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="151">
       <formula>NOT(ISERROR(SEARCH("proofpoint",A1)))</formula>
     </cfRule>
-    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="142">
+    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="152">
       <formula>NOT(ISERROR(SEARCH(" vpn",A1)))</formula>
     </cfRule>
-    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="142">
+    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="152">
       <formula>NOT(ISERROR(SEARCH(" tor",A1)))</formula>
     </cfRule>
-    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="142">
+    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="152">
       <formula>NOT(ISERROR(SEARCH(" proxy",A1)))</formula>
     </cfRule>
-    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="143">
+    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="153">
       <formula>NOT(ISERROR(SEARCH(" hosting",A1)))</formula>
     </cfRule>
-    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="143">
+    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="153">
       <formula>NOT(ISERROR(SEARCH(" cloud",A1)))</formula>
     </cfRule>
-    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="143">
+    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="153">
       <formula>NOT(ISERROR(SEARCH(" datacenter",A1)))</formula>
     </cfRule>
-    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="144">
+    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="154">
       <formula>NOT(ISERROR(SEARCH("mobile",A1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
DEV: Replaced Write-Warning and Write-Verbose with Write-PSFMessage.
</commit_message>
<xml_diff>
--- a/Data/IpAddressConditionalFormattingTemplate.xlsx
+++ b/Data/IpAddressConditionalFormattingTemplate.xlsx
@@ -195,7 +195,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="225">
+  <dxfs count="230">
     <dxf>
       <fill>
         <patternFill>
@@ -262,6 +262,41 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
     <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <fill>
         <patternFill>
@@ -2264,31 +2299,31 @@
     <row r="78" ht="15" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="A:A">
-    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="220">
+    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="225">
       <formula>NOT(ISERROR(SEARCH("microsoft",A1)))</formula>
     </cfRule>
-    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="221">
+    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="226">
       <formula>NOT(ISERROR(SEARCH("proofpoint",A1)))</formula>
     </cfRule>
-    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="222">
+    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="227">
       <formula>NOT(ISERROR(SEARCH(" vpn",A1)))</formula>
     </cfRule>
-    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="222">
+    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="227">
       <formula>NOT(ISERROR(SEARCH(" tor",A1)))</formula>
     </cfRule>
-    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="222">
+    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="227">
       <formula>NOT(ISERROR(SEARCH(" proxy",A1)))</formula>
     </cfRule>
-    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="223">
+    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="228">
       <formula>NOT(ISERROR(SEARCH(" hosting",A1)))</formula>
     </cfRule>
-    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="223">
+    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="228">
       <formula>NOT(ISERROR(SEARCH(" cloud",A1)))</formula>
     </cfRule>
-    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="223">
+    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="228">
       <formula>NOT(ISERROR(SEARCH(" datacenter",A1)))</formula>
     </cfRule>
-    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="224">
+    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="229">
       <formula>NOT(ISERROR(SEARCH("mobile",A1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
DEV: Built module. Updated AGENTS.md. Split off RELEASING.md.
</commit_message>
<xml_diff>
--- a/Data/IpAddressConditionalFormattingTemplate.xlsx
+++ b/Data/IpAddressConditionalFormattingTemplate.xlsx
@@ -195,7 +195,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="230">
+  <dxfs count="240">
     <dxf>
       <fill>
         <patternFill>
@@ -262,6 +262,76 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
     <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <fill>
         <patternFill>
@@ -2299,31 +2369,31 @@
     <row r="78" ht="15" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="A:A">
-    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="225">
+    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="235">
       <formula>NOT(ISERROR(SEARCH("microsoft",A1)))</formula>
     </cfRule>
-    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="226">
+    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="236">
       <formula>NOT(ISERROR(SEARCH("proofpoint",A1)))</formula>
     </cfRule>
-    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="227">
+    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="237">
       <formula>NOT(ISERROR(SEARCH(" vpn",A1)))</formula>
     </cfRule>
-    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="227">
+    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="237">
       <formula>NOT(ISERROR(SEARCH(" tor",A1)))</formula>
     </cfRule>
-    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="227">
+    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="237">
       <formula>NOT(ISERROR(SEARCH(" proxy",A1)))</formula>
     </cfRule>
-    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="228">
+    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="238">
       <formula>NOT(ISERROR(SEARCH(" hosting",A1)))</formula>
     </cfRule>
-    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="228">
+    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="238">
       <formula>NOT(ISERROR(SEARCH(" cloud",A1)))</formula>
     </cfRule>
-    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="228">
+    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="238">
       <formula>NOT(ISERROR(SEARCH(" datacenter",A1)))</formula>
     </cfRule>
-    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="229">
+    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="239">
       <formula>NOT(ISERROR(SEARCH("mobile",A1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
DEV: Updated Install-Dependencies script and built.
</commit_message>
<xml_diff>
--- a/Data/IpAddressConditionalFormattingTemplate.xlsx
+++ b/Data/IpAddressConditionalFormattingTemplate.xlsx
@@ -195,7 +195,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="285">
+  <dxfs count="295">
     <dxf>
       <fill>
         <patternFill>
@@ -262,6 +262,76 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
     <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <fill>
         <patternFill>
@@ -2684,31 +2754,31 @@
     <row r="78" ht="15" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="A:A">
-    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="280">
+    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="290">
       <formula>NOT(ISERROR(SEARCH("microsoft",A1)))</formula>
     </cfRule>
-    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="281">
+    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="291">
       <formula>NOT(ISERROR(SEARCH("proofpoint",A1)))</formula>
     </cfRule>
-    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="282">
+    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="292">
       <formula>NOT(ISERROR(SEARCH(" vpn",A1)))</formula>
     </cfRule>
-    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="282">
+    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="292">
       <formula>NOT(ISERROR(SEARCH(" tor",A1)))</formula>
     </cfRule>
-    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="282">
+    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="292">
       <formula>NOT(ISERROR(SEARCH(" proxy",A1)))</formula>
     </cfRule>
-    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="283">
+    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="293">
       <formula>NOT(ISERROR(SEARCH(" hosting",A1)))</formula>
     </cfRule>
-    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="283">
+    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="293">
       <formula>NOT(ISERROR(SEARCH(" cloud",A1)))</formula>
     </cfRule>
-    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="283">
+    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="293">
       <formula>NOT(ISERROR(SEARCH(" datacenter",A1)))</formula>
     </cfRule>
-    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="284">
+    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="294">
       <formula>NOT(ISERROR(SEARCH("mobile",A1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
chore(build): refresh root module artifacts
Rebuild the root psm1, psd1, Data, and ScriptsToProcess from source so
the built module matches the auth and playbook changes. Includes the
bundled MSAL cache-extension DLL in the built Data folder.
</commit_message>
<xml_diff>
--- a/Data/IpAddressConditionalFormattingTemplate.xlsx
+++ b/Data/IpAddressConditionalFormattingTemplate.xlsx
@@ -195,7 +195,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="310">
+  <dxfs count="325">
     <dxf>
       <fill>
         <patternFill>
@@ -262,6 +262,111 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
     <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <fill>
         <patternFill>
@@ -2859,31 +2964,31 @@
     <row r="78" ht="15" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="A:A">
-    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="305">
+    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="320">
       <formula>NOT(ISERROR(SEARCH("microsoft",A1)))</formula>
     </cfRule>
-    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="306">
+    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="321">
       <formula>NOT(ISERROR(SEARCH("proofpoint",A1)))</formula>
     </cfRule>
-    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="307">
+    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="322">
       <formula>NOT(ISERROR(SEARCH(" vpn",A1)))</formula>
     </cfRule>
-    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="307">
+    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="322">
       <formula>NOT(ISERROR(SEARCH(" tor",A1)))</formula>
     </cfRule>
-    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="307">
+    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="322">
       <formula>NOT(ISERROR(SEARCH(" proxy",A1)))</formula>
     </cfRule>
-    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="308">
+    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="323">
       <formula>NOT(ISERROR(SEARCH(" hosting",A1)))</formula>
     </cfRule>
-    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="308">
+    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="323">
       <formula>NOT(ISERROR(SEARCH(" cloud",A1)))</formula>
     </cfRule>
-    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="308">
+    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="323">
       <formula>NOT(ISERROR(SEARCH(" datacenter",A1)))</formula>
     </cfRule>
-    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="309">
+    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="324">
       <formula>NOT(ISERROR(SEARCH("mobile",A1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
chore: moved files. new build
</commit_message>
<xml_diff>
--- a/Data/IpAddressConditionalFormattingTemplate.xlsx
+++ b/Data/IpAddressConditionalFormattingTemplate.xlsx
@@ -195,7 +195,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="310">
+  <dxfs count="330">
     <dxf>
       <fill>
         <patternFill>
@@ -262,6 +262,146 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
     <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <fill>
         <patternFill>
@@ -2859,31 +2999,31 @@
     <row r="78" ht="15" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="A:A">
-    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="305">
+    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="325">
       <formula>NOT(ISERROR(SEARCH("microsoft",A1)))</formula>
     </cfRule>
-    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="306">
+    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="326">
       <formula>NOT(ISERROR(SEARCH("proofpoint",A1)))</formula>
     </cfRule>
-    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="307">
+    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="327">
       <formula>NOT(ISERROR(SEARCH(" vpn",A1)))</formula>
     </cfRule>
-    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="307">
+    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="327">
       <formula>NOT(ISERROR(SEARCH(" tor",A1)))</formula>
     </cfRule>
-    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="307">
+    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="327">
       <formula>NOT(ISERROR(SEARCH(" proxy",A1)))</formula>
     </cfRule>
-    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="308">
+    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="328">
       <formula>NOT(ISERROR(SEARCH(" hosting",A1)))</formula>
     </cfRule>
-    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="308">
+    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="328">
       <formula>NOT(ISERROR(SEARCH(" cloud",A1)))</formula>
     </cfRule>
-    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="308">
+    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="328">
       <formula>NOT(ISERROR(SEARCH(" datacenter",A1)))</formula>
     </cfRule>
-    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="309">
+    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="329">
       <formula>NOT(ISERROR(SEARCH("mobile",A1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
chore: drop built module artifacts from PR
The merge into develop conflicted on generated root-level build output.
Per AGENTS.md, root *.psm1/*.psd1, ScriptsToProcess/, and Data/ are built
from Source/ and should not be hand-committed. Reset those root artifacts
and Tests.ps1 to develop, and remove the generated root copy of the MSAL
cache-extension DLL. The source-of-truth assets under Source/ (including
Source/Data/Microsoft.Identity.Client.Extensions.Msal.dll) are unchanged,
so a rebuild regenerates the root output.
</commit_message>
<xml_diff>
--- a/Data/IpAddressConditionalFormattingTemplate.xlsx
+++ b/Data/IpAddressConditionalFormattingTemplate.xlsx
@@ -195,7 +195,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="325">
+  <dxfs count="350">
     <dxf>
       <fill>
         <patternFill>
@@ -262,6 +262,181 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
     <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <fill>
         <patternFill>
@@ -2964,31 +3139,31 @@
     <row r="78" ht="15" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="A:A">
-    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="320">
+    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="345">
       <formula>NOT(ISERROR(SEARCH("microsoft",A1)))</formula>
     </cfRule>
-    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="321">
+    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="346">
       <formula>NOT(ISERROR(SEARCH("proofpoint",A1)))</formula>
     </cfRule>
-    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="322">
+    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="347">
       <formula>NOT(ISERROR(SEARCH(" vpn",A1)))</formula>
     </cfRule>
-    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="322">
+    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="347">
       <formula>NOT(ISERROR(SEARCH(" tor",A1)))</formula>
     </cfRule>
-    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="322">
+    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="347">
       <formula>NOT(ISERROR(SEARCH(" proxy",A1)))</formula>
     </cfRule>
-    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="323">
+    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="348">
       <formula>NOT(ISERROR(SEARCH(" hosting",A1)))</formula>
     </cfRule>
-    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="323">
+    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="348">
       <formula>NOT(ISERROR(SEARCH(" cloud",A1)))</formula>
     </cfRule>
-    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="323">
+    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="348">
       <formula>NOT(ISERROR(SEARCH(" datacenter",A1)))</formula>
     </cfRule>
-    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="324">
+    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="349">
       <formula>NOT(ISERROR(SEARCH("mobile",A1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Sync remaining working-tree changes
Commit the leftover uncommitted changes so the working tree is clean. These
are unrelated to the chunking fix and are grouped only to clear the tree:

- auth-related: M365IncidentResponseTools.psd1/.psm1, Data/ConfigTemplate.json,
  ScriptsToProcess/Confirm-Dependencies.ps1, and the new
  Microsoft.Identity.Client.Extensions.Msal.dll dependency.
- data files: IpAddressConditionalFormattingTemplate.xlsx (Data + Source/Data)
  and Source/Data/UALAllOperations.xlsx (updated by a test run).
- in-progress edits to tests/Pester/Get-IRTUnifiedAuditLog.Paths.Online.Tests.ps1.
</commit_message>
<xml_diff>
--- a/Data/IpAddressConditionalFormattingTemplate.xlsx
+++ b/Data/IpAddressConditionalFormattingTemplate.xlsx
@@ -195,7 +195,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="350">
+  <dxfs count="360">
     <dxf>
       <fill>
         <patternFill>
@@ -262,6 +262,76 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
     <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <fill>
         <patternFill>
@@ -3139,31 +3209,31 @@
     <row r="78" ht="15" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="A:A">
-    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="345">
+    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="355">
       <formula>NOT(ISERROR(SEARCH("microsoft",A1)))</formula>
     </cfRule>
-    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="346">
+    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="356">
       <formula>NOT(ISERROR(SEARCH("proofpoint",A1)))</formula>
     </cfRule>
-    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="347">
+    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="357">
       <formula>NOT(ISERROR(SEARCH(" vpn",A1)))</formula>
     </cfRule>
-    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="347">
+    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="357">
       <formula>NOT(ISERROR(SEARCH(" tor",A1)))</formula>
     </cfRule>
-    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="347">
+    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="357">
       <formula>NOT(ISERROR(SEARCH(" proxy",A1)))</formula>
     </cfRule>
-    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="348">
+    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="358">
       <formula>NOT(ISERROR(SEARCH(" hosting",A1)))</formula>
     </cfRule>
-    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="348">
+    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="358">
       <formula>NOT(ISERROR(SEARCH(" cloud",A1)))</formula>
     </cfRule>
-    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="348">
+    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="358">
       <formula>NOT(ISERROR(SEARCH(" datacenter",A1)))</formula>
     </cfRule>
-    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="349">
+    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="359">
       <formula>NOT(ISERROR(SEARCH("mobile",A1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
chore: updated build artifacts.
</commit_message>
<xml_diff>
--- a/Data/IpAddressConditionalFormattingTemplate.xlsx
+++ b/Data/IpAddressConditionalFormattingTemplate.xlsx
@@ -195,7 +195,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="360">
+  <dxfs count="375">
     <dxf>
       <fill>
         <patternFill>
@@ -262,6 +262,111 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
     <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <fill>
         <patternFill>
@@ -3209,31 +3314,31 @@
     <row r="78" ht="15" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="A:A">
-    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="355">
+    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="370">
       <formula>NOT(ISERROR(SEARCH("microsoft",A1)))</formula>
     </cfRule>
-    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="356">
+    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="371">
       <formula>NOT(ISERROR(SEARCH("proofpoint",A1)))</formula>
     </cfRule>
-    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="357">
+    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="372">
       <formula>NOT(ISERROR(SEARCH(" vpn",A1)))</formula>
     </cfRule>
-    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="357">
+    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="372">
       <formula>NOT(ISERROR(SEARCH(" tor",A1)))</formula>
     </cfRule>
-    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="357">
+    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="372">
       <formula>NOT(ISERROR(SEARCH(" proxy",A1)))</formula>
     </cfRule>
-    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="358">
+    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="373">
       <formula>NOT(ISERROR(SEARCH(" hosting",A1)))</formula>
     </cfRule>
-    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="358">
+    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="373">
       <formula>NOT(ISERROR(SEARCH(" cloud",A1)))</formula>
     </cfRule>
-    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="358">
+    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="373">
       <formula>NOT(ISERROR(SEARCH(" datacenter",A1)))</formula>
     </cfRule>
-    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="359">
+    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="374">
       <formula>NOT(ISERROR(SEARCH("mobile",A1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Added -DeviceCode option to Get-IRTEntraSigninlog.
</commit_message>
<xml_diff>
--- a/Data/IpAddressConditionalFormattingTemplate.xlsx
+++ b/Data/IpAddressConditionalFormattingTemplate.xlsx
@@ -195,7 +195,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="380">
+  <dxfs count="385">
     <dxf>
       <fill>
         <patternFill>
@@ -262,6 +262,41 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
     <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <fill>
         <patternFill>
@@ -3349,31 +3384,31 @@
     <row r="78" ht="15" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="A:A">
-    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="375">
+    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="380">
       <formula>NOT(ISERROR(SEARCH("microsoft",A1)))</formula>
     </cfRule>
-    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="376">
+    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="381">
       <formula>NOT(ISERROR(SEARCH("proofpoint",A1)))</formula>
     </cfRule>
-    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="377">
+    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="382">
       <formula>NOT(ISERROR(SEARCH(" vpn",A1)))</formula>
     </cfRule>
-    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="377">
+    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="382">
       <formula>NOT(ISERROR(SEARCH(" tor",A1)))</formula>
     </cfRule>
-    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="377">
+    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="382">
       <formula>NOT(ISERROR(SEARCH(" proxy",A1)))</formula>
     </cfRule>
-    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="378">
+    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="383">
       <formula>NOT(ISERROR(SEARCH(" hosting",A1)))</formula>
     </cfRule>
-    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="378">
+    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="383">
       <formula>NOT(ISERROR(SEARCH(" cloud",A1)))</formula>
     </cfRule>
-    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="378">
+    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="383">
       <formula>NOT(ISERROR(SEARCH(" datacenter",A1)))</formula>
     </cfRule>
-    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="379">
+    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="384">
       <formula>NOT(ISERROR(SEARCH("mobile",A1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
chore: rebuild module artifacts for v2.10.0 release verification
Rebuilt root .psm1 and IP conditional-formatting templates via Build.ps1
during the release procedure. No source changes.
</commit_message>
<xml_diff>
--- a/Data/IpAddressConditionalFormattingTemplate.xlsx
+++ b/Data/IpAddressConditionalFormattingTemplate.xlsx
@@ -195,7 +195,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="410">
+  <dxfs count="420">
     <dxf>
       <fill>
         <patternFill>
@@ -262,6 +262,76 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
     <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <fill>
         <patternFill>
@@ -3559,31 +3629,31 @@
     <row r="78" ht="15" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="A:A">
-    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="405">
+    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="415">
       <formula>NOT(ISERROR(SEARCH("microsoft",A1)))</formula>
     </cfRule>
-    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="406">
+    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="416">
       <formula>NOT(ISERROR(SEARCH("proofpoint",A1)))</formula>
     </cfRule>
-    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="407">
+    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="417">
       <formula>NOT(ISERROR(SEARCH(" vpn",A1)))</formula>
     </cfRule>
-    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="407">
+    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="417">
       <formula>NOT(ISERROR(SEARCH(" tor",A1)))</formula>
     </cfRule>
-    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="407">
+    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="417">
       <formula>NOT(ISERROR(SEARCH(" proxy",A1)))</formula>
     </cfRule>
-    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="408">
+    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="418">
       <formula>NOT(ISERROR(SEARCH(" hosting",A1)))</formula>
     </cfRule>
-    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="408">
+    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="418">
       <formula>NOT(ISERROR(SEARCH(" cloud",A1)))</formula>
     </cfRule>
-    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="408">
+    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="418">
       <formula>NOT(ISERROR(SEARCH(" datacenter",A1)))</formula>
     </cfRule>
-    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="409">
+    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="419">
       <formula>NOT(ISERROR(SEARCH("mobile",A1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
fix: removed import of PSFramework because it's not available when running onprem functions remotely.
</commit_message>
<xml_diff>
--- a/Data/IpAddressConditionalFormattingTemplate.xlsx
+++ b/Data/IpAddressConditionalFormattingTemplate.xlsx
@@ -195,7 +195,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="420">
+  <dxfs count="430">
     <dxf>
       <fill>
         <patternFill>
@@ -262,6 +262,76 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
     <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <fill>
         <patternFill>
@@ -3629,31 +3699,31 @@
     <row r="78" ht="15" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="A:A">
-    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="415">
+    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="425">
       <formula>NOT(ISERROR(SEARCH("microsoft",A1)))</formula>
     </cfRule>
-    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="416">
+    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="426">
       <formula>NOT(ISERROR(SEARCH("proofpoint",A1)))</formula>
     </cfRule>
-    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="417">
+    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="427">
       <formula>NOT(ISERROR(SEARCH(" vpn",A1)))</formula>
     </cfRule>
-    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="417">
+    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="427">
       <formula>NOT(ISERROR(SEARCH(" tor",A1)))</formula>
     </cfRule>
-    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="417">
+    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="427">
       <formula>NOT(ISERROR(SEARCH(" proxy",A1)))</formula>
     </cfRule>
-    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="418">
+    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="428">
       <formula>NOT(ISERROR(SEARCH(" hosting",A1)))</formula>
     </cfRule>
-    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="418">
+    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="428">
       <formula>NOT(ISERROR(SEARCH(" cloud",A1)))</formula>
     </cfRule>
-    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="418">
+    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="428">
       <formula>NOT(ISERROR(SEARCH(" datacenter",A1)))</formula>
     </cfRule>
-    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="419">
+    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="429">
       <formula>NOT(ISERROR(SEARCH("mobile",A1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
build: rebuild the module from Source
Picks up the dependency-script rename, the RequiredModules.psd1 declaration,
and the banner change that were only in Source/ until now. The plural
Confirm-Dependencies.ps1 and Install-Dependencies.ps1 are gone from the
module root because Source/ no longer has them.

Build.ps1's PreBuild step rewrites the IP address conditional formatting
template, so both copies move together.

The detect-secrets baseline records a new line number for an
already-audited, non-secret match that shifted when the psm1 was rebuilt.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/IpAddressConditionalFormattingTemplate.xlsx
+++ b/Data/IpAddressConditionalFormattingTemplate.xlsx
@@ -195,7 +195,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="430">
+  <dxfs count="435">
     <dxf>
       <fill>
         <patternFill>
@@ -262,6 +262,41 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
     <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <fill>
         <patternFill>
@@ -3699,31 +3734,31 @@
     <row r="78" ht="15" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="A:A">
-    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="425">
+    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="430">
       <formula>NOT(ISERROR(SEARCH("microsoft",A1)))</formula>
     </cfRule>
-    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="426">
+    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="431">
       <formula>NOT(ISERROR(SEARCH("proofpoint",A1)))</formula>
     </cfRule>
-    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="427">
+    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="432">
       <formula>NOT(ISERROR(SEARCH(" vpn",A1)))</formula>
     </cfRule>
-    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="427">
+    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="432">
       <formula>NOT(ISERROR(SEARCH(" tor",A1)))</formula>
     </cfRule>
-    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="427">
+    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="432">
       <formula>NOT(ISERROR(SEARCH(" proxy",A1)))</formula>
     </cfRule>
-    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="428">
+    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="433">
       <formula>NOT(ISERROR(SEARCH(" hosting",A1)))</formula>
     </cfRule>
-    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="428">
+    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="433">
       <formula>NOT(ISERROR(SEARCH(" cloud",A1)))</formula>
     </cfRule>
-    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="428">
+    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="433">
       <formula>NOT(ISERROR(SEARCH(" datacenter",A1)))</formula>
     </cfRule>
-    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="429">
+    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="434">
       <formula>NOT(ISERROR(SEARCH("mobile",A1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
build: rebuild module artifacts for v2.11.0
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/IpAddressConditionalFormattingTemplate.xlsx
+++ b/Data/IpAddressConditionalFormattingTemplate.xlsx
@@ -195,7 +195,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="440">
+  <dxfs count="455">
     <dxf>
       <fill>
         <patternFill>
@@ -262,6 +262,111 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
     <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <fill>
         <patternFill>
@@ -3769,31 +3874,31 @@
     <row r="78" ht="15" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="A:A">
-    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="435">
+    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="450">
       <formula>NOT(ISERROR(SEARCH("microsoft",A1)))</formula>
     </cfRule>
-    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="436">
+    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="451">
       <formula>NOT(ISERROR(SEARCH("proofpoint",A1)))</formula>
     </cfRule>
-    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="437">
+    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="452">
       <formula>NOT(ISERROR(SEARCH(" vpn",A1)))</formula>
     </cfRule>
-    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="437">
+    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="452">
       <formula>NOT(ISERROR(SEARCH(" tor",A1)))</formula>
     </cfRule>
-    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="437">
+    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="452">
       <formula>NOT(ISERROR(SEARCH(" proxy",A1)))</formula>
     </cfRule>
-    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="438">
+    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="453">
       <formula>NOT(ISERROR(SEARCH(" hosting",A1)))</formula>
     </cfRule>
-    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="438">
+    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="453">
       <formula>NOT(ISERROR(SEARCH(" cloud",A1)))</formula>
     </cfRule>
-    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="438">
+    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="453">
       <formula>NOT(ISERROR(SEARCH(" datacenter",A1)))</formula>
     </cfRule>
-    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="439">
+    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="454">
       <formula>NOT(ISERROR(SEARCH("mobile",A1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
build: rebuild module artifacts
Exports Get-IRTTeamsExternalDomain and its aliases from the manifest,
and picks up the conditional-formatting template PreBuild regenerates on
every build.

The detect-secrets baseline moves with the rebuilt psm1: line numbers
only, no new or changed findings.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/IpAddressConditionalFormattingTemplate.xlsx
+++ b/Data/IpAddressConditionalFormattingTemplate.xlsx
@@ -195,7 +195,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="455">
+  <dxfs count="465">
     <dxf>
       <fill>
         <patternFill>
@@ -262,6 +262,76 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
     <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <fill>
         <patternFill>
@@ -3874,31 +3944,31 @@
     <row r="78" ht="15" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="A:A">
-    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="450">
+    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="460">
       <formula>NOT(ISERROR(SEARCH("microsoft",A1)))</formula>
     </cfRule>
-    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="451">
+    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="461">
       <formula>NOT(ISERROR(SEARCH("proofpoint",A1)))</formula>
     </cfRule>
-    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="452">
+    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="462">
       <formula>NOT(ISERROR(SEARCH(" vpn",A1)))</formula>
     </cfRule>
-    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="452">
+    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="462">
       <formula>NOT(ISERROR(SEARCH(" tor",A1)))</formula>
     </cfRule>
-    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="452">
+    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="462">
       <formula>NOT(ISERROR(SEARCH(" proxy",A1)))</formula>
     </cfRule>
-    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="453">
+    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="463">
       <formula>NOT(ISERROR(SEARCH(" hosting",A1)))</formula>
     </cfRule>
-    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="453">
+    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="463">
       <formula>NOT(ISERROR(SEARCH(" cloud",A1)))</formula>
     </cfRule>
-    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="453">
+    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="463">
       <formula>NOT(ISERROR(SEARCH(" datacenter",A1)))</formula>
     </cfRule>
-    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="454">
+    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="464">
       <formula>NOT(ISERROR(SEARCH("mobile",A1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>